<commit_message>
added more tests to NC and more code to seniorNM functionality
</commit_message>
<xml_diff>
--- a/src/data/excel-mockdata-NY-medFeil/pamelding_Ålesund_Turn.xlsx
+++ b/src/data/excel-mockdata-NY-medFeil/pamelding_Ålesund_Turn.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="52">
   <si>
     <t>Påmelding Norges cup Turn menn</t>
   </si>
@@ -161,9 +161,6 @@
     <t>Anders Svendsen</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Jonas Karlsen</t>
   </si>
   <si>
@@ -183,7 +180,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm-dd-yyyy"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -227,6 +224,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Consolas"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -345,7 +348,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -416,7 +419,7 @@
     <xf xfId="0" numFmtId="0" borderId="7" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="7" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
@@ -459,9 +462,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -781,32 +781,32 @@
   <dimension ref="A1:Z1001"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="40" width="24.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="42" width="5.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="42" width="11.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="42" width="5.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="42" width="5.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="40" width="12.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="42" width="17.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="43" width="12.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="42" width="10.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="42" width="7.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="42" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="42" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="39" width="24.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="40" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="41" width="5.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="41" width="11.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="41" width="5.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="41" width="5.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="39" width="12.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="41" width="17.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="42" width="12.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="41" width="10.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="41" width="7.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="41" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="41" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="44.25">
@@ -1262,7 +1262,7 @@
         <v>41</v>
       </c>
       <c r="B12" s="35">
-        <v>2013</v>
+        <v>25569.041689965277</v>
       </c>
       <c r="C12" s="36" t="s">
         <v>39</v>
@@ -1310,7 +1310,7 @@
         <v>39</v>
       </c>
       <c r="B13" s="38">
-        <v>41640</v>
+        <v>25569.041689976853</v>
       </c>
       <c r="C13" s="36" t="s">
         <v>39</v>
@@ -1356,7 +1356,7 @@
         <v>42</v>
       </c>
       <c r="B14" s="35">
-        <v>41640</v>
+        <v>25569.041689976853</v>
       </c>
       <c r="C14" s="36" t="s">
         <v>39</v>
@@ -1448,7 +1448,7 @@
         <v>44</v>
       </c>
       <c r="B16" s="35">
-        <v>41640.00069444445</v>
+        <v>25569.041689976853</v>
       </c>
       <c r="C16" s="36" t="s">
         <v>39</v>
@@ -1494,7 +1494,7 @@
         <v>45</v>
       </c>
       <c r="B17" s="35">
-        <v>40544.00069444445</v>
+        <v>25569.04168994213</v>
       </c>
       <c r="C17" s="36"/>
       <c r="D17" s="36" t="s">
@@ -1542,7 +1542,7 @@
         <v>46</v>
       </c>
       <c r="B18" s="35">
-        <v>2011</v>
+        <v>25569.04168994213</v>
       </c>
       <c r="C18" s="36"/>
       <c r="D18" s="36" t="s">
@@ -1590,9 +1590,7 @@
       <c r="B19" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="39" t="s">
-        <v>48</v>
-      </c>
+      <c r="C19" s="36"/>
       <c r="D19" s="36"/>
       <c r="E19" s="36"/>
       <c r="F19" s="36"/>
@@ -1631,14 +1629,12 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="34" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B20" s="35">
-        <v>2010</v>
+        <v>25569.041689930556</v>
       </c>
-      <c r="C20" s="39" t="s">
-        <v>48</v>
-      </c>
+      <c r="C20" s="36"/>
       <c r="D20" s="36"/>
       <c r="E20" s="36" t="s">
         <v>39</v>
@@ -1679,10 +1675,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="34" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B21" s="35">
-        <v>2007</v>
+        <v>25569.041689895832</v>
       </c>
       <c r="C21" s="36"/>
       <c r="D21" s="36"/>
@@ -1725,10 +1721,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="34" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B22" s="35">
-        <v>2007</v>
+        <v>25569.041689895832</v>
       </c>
       <c r="C22" s="36"/>
       <c r="D22" s="36"/>
@@ -1769,10 +1765,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="34" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B23" s="35">
-        <v>1994</v>
+        <v>25569.04168974537</v>
       </c>
       <c r="C23" s="36"/>
       <c r="D23" s="36"/>

</xml_diff>